<commit_message>
Re audit pause resume
</commit_message>
<xml_diff>
--- a/docs/qc/testcases/UC-EXBOT-pause-resume/UC-EXBOT-pause-resume_testcases_20260706_v5.xlsx
+++ b/docs/qc/testcases/UC-EXBOT-pause-resume/UC-EXBOT-pause-resume_testcases_20260706_v5.xlsx
@@ -15447,12 +15447,19 @@
       </c>
       <c r="D5" s="114" t="inlineStr">
         <is>
-          <t>Send a pause request for the bot.</t>
+          <t>1. Send POST /api/exbot/pause with botId.
+2. Lambda verifies status='active' and lifecycle_state='active'.
+3. Lambda executes conditional UPDATE: bots.status='paused' WHERE bot_id=X AND status='active'.
+4. Returns HTTP 200 + MSG-SUC-81.</t>
         </is>
       </c>
       <c r="E5" s="114" t="inlineStr">
         <is>
-          <t>The status changes to 'paused' in Aurora PostgreSQL. The lifecycle_state stays unchanged. The hedge leg size and LP NFT token ID stay unchanged. The API returns HTTP 200 with the message matching MSG-SUC-81. (Reference: UC §3, FR-EXBOT-005, BR-EXBOT-002.)</t>
+          <t>1. bots.status='paused'.
+2. bots.lifecycle_state='active' (unchanged).
+3. hedge_legs.last_known_hl_short_size unchanged.
+4. positions.token_id unchanged.
+5. API returns HTTP 200 with message 'Bot paused. Hedge and LP are maintained.' (Reference: UC §3, FR-EXBOT-005, BR-EXBOT-002.)</t>
         </is>
       </c>
       <c r="F5" s="114" t="inlineStr">
@@ -15479,12 +15486,19 @@
       </c>
       <c r="D6" s="114" t="inlineStr">
         <is>
-          <t>Send a pause request for the bot in safe_mode.</t>
+          <t>1. Send POST /api/exbot/pause with botId.
+2. Lambda queries Aurora: bots.status='safe_mode'.
+3. Lambda skips UPDATE (blocked).
+4. Returns HTTP 409 + E-EXBOT-013.</t>
         </is>
       </c>
       <c r="E6" s="114" t="inlineStr">
         <is>
-          <t>The request is rejected and the status stays 'safe_mode'. The API returns HTTP 409 with the message "Bot is in Safe Mode. You can close the bot instead." (E-EXBOT-013). (Reference: UC §5 A1, FR-EXBOT-050.)</t>
+          <t>1. Request rejected.
+2. bots.status stays 'safe_mode' (unchanged).
+3. API returns HTTP 409 with 'Bot is in Safe Mode. You can close the bot instead.' (E-EXBOT-013).
+4. No audit log entry for failed pause attempt.
+(Reference: UC §5 A1, FR-EXBOT-050.)</t>
         </is>
       </c>
       <c r="F6" s="114" t="inlineStr">
@@ -15511,12 +15525,19 @@
       </c>
       <c r="D7" s="114" t="inlineStr">
         <is>
-          <t>Send another pause request for the already-paused bot.</t>
+          <t>1. Send POST /api/exbot/pause with botId.
+2. Lambda queries Aurora: bots.status='paused'.
+3. Conditional UPDATE finds no match (WHERE status='active').
+4. Returns HTTP 200 + 'Bot already paused. No change needed.'</t>
         </is>
       </c>
       <c r="E7" s="114" t="inlineStr">
         <is>
-          <t>The request succeeds with no state change (idempotent). The API returns HTTP 200 with the message "Bot already paused. No change needed." Aurora PostgreSQL is not modified by the second request. (Reference: UC §5 A3, FR-EXBOT-005.)</t>
+          <t>1. No state change.
+2. bots.updated_at unchanged (no actual UPDATE).
+3. API returns HTTP 200 with 'Bot already paused. No change needed.'
+4. No new audit log entry.
+(Reference: UC §5 A3, FR-EXBOT-005.)</t>
         </is>
       </c>
       <c r="F7" s="114" t="inlineStr">
@@ -15543,12 +15564,20 @@
       </c>
       <c r="D8" s="114" t="inlineStr">
         <is>
-          <t>Send a pause request for the bot with the non-active lifecycle_state.</t>
+          <t>1. Send POST /api/exbot/pause with botId.
+2. Lambda queries Aurora: bots.lifecycle_state is non-active.
+3. Lambda skips UPDATE.
+4. Returns HTTP 409 with error message.</t>
         </is>
       </c>
       <c r="E8" s="114" t="inlineStr">
         <is>
-          <t>The request is rejected and the status stays 'active'. The API returns HTTP 409 with an error message. Only lifecycle_state='active' can be paused per BA decision (Q7, 2026-07-03). (Reference: UC §2, states.md.)</t>
+          <t>1. Request rejected.
+2. bots.status='active' (unchanged).
+3. bots.lifecycle_state unchanged.
+4. API returns HTTP 409.
+Only lifecycle_state='active' can be paused per BA decision (Q7, 2026-07-03).
+(Reference: UC §2, states.md.)</t>
         </is>
       </c>
       <c r="F8" s="114" t="inlineStr">
@@ -15575,12 +15604,20 @@
       </c>
       <c r="D9" s="114" t="inlineStr">
         <is>
-          <t>Send two pause requests at the same time for the same bot.</t>
+          <t>1. Terminal 1: Send POST /api/exbot/pause.
+2. Terminal 2: Send POST /api/exbot/pause at same time.
+3. Lambda 1 executes conditional UPDATE -&gt; MATCH -&gt; updates to 'paused'.
+4. Lambda 2 executes conditional UPDATE -&gt; NO MATCH -&gt; returns idempotent success.</t>
         </is>
       </c>
       <c r="E9" s="114" t="inlineStr">
         <is>
-          <t>Exactly one state change occurs. The first request wins and changes status to 'paused'. The second request finds status='paused' and returns the idempotent success message. No error, no partial state, no race condition. (Reference: UC §5 A3, Q3 resolved.)</t>
+          <t>1. Exactly 1 state change occurs.
+2. Request 1 returns 'Bot paused. Hedge and LP are maintained.'
+3. Request 2 returns 'Bot already paused. No change needed.'
+4. Only 1 audit log entry.
+5. No partial state, no race condition.
+(Reference: UC §5 A3, Q3 resolved.)</t>
         </is>
       </c>
       <c r="F9" s="114" t="inlineStr">
@@ -15607,12 +15644,15 @@
       </c>
       <c r="D10" s="114" t="inlineStr">
         <is>
-          <t>Send a pause request and capture the API response body.</t>
+          <t>1. Send POST /api/exbot/pause with botId.
+2. Capture API response body.</t>
         </is>
       </c>
       <c r="E10" s="114" t="inlineStr">
         <is>
-          <t>The response body contains the message "Bot paused. Hedge and LP are maintained." matching MSG-SUC-81 from message-list.md §MSG-EXBOT. (Reference: UC §3 step 7, message-list.md, Q9 resolved.)</t>
+          <t>1. Response body contains message: 'Bot paused. Hedge and LP are maintained.' exactly matching MSG-SUC-81.
+2. No extra spaces, no typos.
+(Reference: UC §3 step 7, message-list.md, Q9 resolved.)</t>
         </is>
       </c>
       <c r="F10" s="114" t="inlineStr">
@@ -15651,12 +15691,16 @@
       </c>
       <c r="D12" s="114" t="inlineStr">
         <is>
-          <t>Send a pause request for the bot. Read the audit log for the latest entry.</t>
+          <t>1. Send POST /api/exbot/pause.
+2. Query audit_log WHERE bot_id=X ORDER BY created_at DESC LIMIT 1.</t>
         </is>
       </c>
       <c r="E12" s="114" t="inlineStr">
         <is>
-          <t>The audit log contains an entry with the action "Bot paused by investor", the bot ID, the user ID, and a timestamp matching the pause time. (Reference: UC §7 Postconditions.)</t>
+          <t>1. Audit log entry exists with action='Bot paused by investor'.
+2. bot_id and user_wallet_address correct.
+3. created_at timestamp matches pause time.
+(Reference: UC §7 Postconditions.)</t>
         </is>
       </c>
       <c r="F12" s="114" t="inlineStr">
@@ -15683,12 +15727,16 @@
       </c>
       <c r="D13" s="114" t="inlineStr">
         <is>
-          <t>Record the current hedge leg size. Send a pause request. Read the hedge leg size again.</t>
+          <t>1. Record hedge_legs.last_known_hl_short_size.
+2. Send POST /api/exbot/pause.
+3. Read hedge_legs.last_known_hl_short_size again.</t>
         </is>
       </c>
       <c r="E13" s="114" t="inlineStr">
         <is>
-          <t>The hedge leg size is exactly the same before and after pause. No HL order is submitted during the pause operation. (Reference: UC §3 step 5, BR-EXBOT-002.)</t>
+          <t>1. Hedge leg size exactly the same before and after pause.
+2. No HL order submitted during pause operation.
+(Reference: UC §3 step 5, BR-EXBOT-002.)</t>
         </is>
       </c>
       <c r="F13" s="114" t="inlineStr">
@@ -15715,12 +15763,16 @@
       </c>
       <c r="D14" s="114" t="inlineStr">
         <is>
-          <t>Record the current LP NFT token ID. Send a pause request. Read the token ID again.</t>
+          <t>1. Record positions.token_id.
+2. Send POST /api/exbot/pause.
+3. Read positions.token_id again.</t>
         </is>
       </c>
       <c r="E14" s="114" t="inlineStr">
         <is>
-          <t>The LP NFT token ID is exactly the same before and after pause. No vault transaction is submitted during the pause operation. (Reference: UC §3 step 6, BR-EXBOT-002.)</t>
+          <t>1. LP NFT token ID exactly the same before and after pause.
+2. No vault transaction submitted during pause operation.
+(Reference: UC §3 step 6, BR-EXBOT-002.)</t>
         </is>
       </c>
       <c r="F14" s="114" t="inlineStr">
@@ -15747,12 +15799,16 @@
       </c>
       <c r="D15" s="114" t="inlineStr">
         <is>
-          <t>Send a pause request while tracking HL API calls.</t>
+          <t>1. Start HL API monitoring.
+2. Send POST /api/exbot/pause.
+3. Check HL API logs for bot's pause timeframe.</t>
         </is>
       </c>
       <c r="E15" s="114" t="inlineStr">
         <is>
-          <t>Zero HL API calls are made during the pause operation. The pause relies solely on Aurora PostgreSQL state. (Reference: UC §3, BR-EXBOT-003.)</t>
+          <t>1. Zero HL API calls during pause operation.
+2. Pause relies solely on Aurora PostgreSQL state.
+(Reference: UC §3, BR-EXBOT-003.)</t>
         </is>
       </c>
       <c r="F15" s="114" t="inlineStr">
@@ -15791,12 +15847,16 @@
       </c>
       <c r="D17" s="114" t="inlineStr">
         <is>
-          <t>Send a pause request but simulate a Lambda crash before the transaction commits.</t>
+          <t>1. Send POST /api/exbot/pause.
+2. Simulate Lambda crash before transaction commits.
+3. Query Aurora PostgreSQL.</t>
         </is>
       </c>
       <c r="E17" s="114" t="inlineStr">
         <is>
-          <t>Aurora PostgreSQL stays in the previous consistent state (status='active'). No partial or inconsistent status value is left in the database. (Reference: Q3 resolved.)</t>
+          <t>1. Aurora PostgreSQL stays at previous consistent state (bots.status='active').
+2. No partial or inconsistent status value left in database.
+(Reference: Q3 resolved.)</t>
         </is>
       </c>
       <c r="F17" s="114" t="inlineStr">
@@ -15847,12 +15907,22 @@
       </c>
       <c r="D20" s="114" t="inlineStr">
         <is>
-          <t>Send a resume request for the bot.</t>
+          <t>1. Send POST /api/exbot/resume with botId.
+2. Lambda verifies bots.status='paused'.
+3. Lambda executes conditional UPDATE: bots.status='active' WHERE bot_id=X AND status='paused'.
+4. Lambda sets next_light_check_at=now+5min+jitter(−45s,+45s).
+5. Lambda enqueues light-check message.
+6. Returns HTTP 200 + MSG-SUC-82.</t>
         </is>
       </c>
       <c r="E20" s="114" t="inlineStr">
         <is>
-          <t>The status changes back to 'active' in Aurora PostgreSQL. The lifecycle_state stays unchanged. The next_light_check_at is set to now plus 5 minutes plus random jitter of minus 45 to plus 45 seconds. A light-check message is enqueued. The API returns HTTP 200 with MSG-SUC-82. (Reference: UC §4, FR-EXBOT-013.)</t>
+          <t>1. bots.status='active'.
+2. bots.lifecycle_state='active' (unchanged).
+3. next_light_check_at set to now+4:15 to 5:45.
+4. light-check message enqueued.
+5. API returns HTTP 200 with 'Bot resumed. Monitoring will resume shortly.'
+(Reference: UC §4, FR-EXBOT-013.)</t>
         </is>
       </c>
       <c r="F20" s="114" t="inlineStr">
@@ -15879,12 +15949,18 @@
       </c>
       <c r="D21" s="114" t="inlineStr">
         <is>
-          <t>Send a resume request for the already-active bot.</t>
+          <t>1. Send POST /api/exbot/resume with botId.
+2. Lambda queries Aurora: bots.status='active'.
+3. Conditional UPDATE finds no match.
+4. Returns HTTP 200 + 'Bot already active. No change needed.'</t>
         </is>
       </c>
       <c r="E21" s="114" t="inlineStr">
         <is>
-          <t>The request succeeds with no state change (idempotent). The API returns HTTP 200 with "Bot already active. No change needed." Aurora PostgreSQL is not modified. (Reference: UC §5 A2, FR-EXBOT-005.)</t>
+          <t>1. No state change.
+2. Aurora PostgreSQL not modified.
+3. API returns HTTP 200 with 'Bot already active. No change needed.'
+(Reference: UC §5 A2, FR-EXBOT-005.)</t>
         </is>
       </c>
       <c r="F21" s="114" t="inlineStr">
@@ -15911,12 +15987,17 @@
       </c>
       <c r="D22" s="114" t="inlineStr">
         <is>
-          <t>Send a resume request with a non-existent bot ID.</t>
+          <t>1. Send POST /api/exbot/resume with non-existent botId.
+2. Lambda queries Aurora: no row found.
+3. Returns HTTP 404.</t>
         </is>
       </c>
       <c r="E22" s="114" t="inlineStr">
         <is>
-          <t>The request is rejected. The API returns HTTP 404 with an error message indicating the bot was not found. (Reference: UC §2.)</t>
+          <t>1. Request rejected.
+2. API returns HTTP 404 with error message indicating bot not found.
+3. No audit log entry created.
+(Reference: UC §2.)</t>
         </is>
       </c>
       <c r="F22" s="114" t="inlineStr">
@@ -15943,12 +16024,17 @@
       </c>
       <c r="D23" s="114" t="inlineStr">
         <is>
-          <t>Record the current time. Send a resume request. Read the next_light_check_at value.</t>
+          <t>1. Record current time.
+2. Send POST /api/exbot/resume.
+3. Read bot_runtime_state.next_light_check_at.
+4. Calculate delta from recorded time.</t>
         </is>
       </c>
       <c r="E23" s="114" t="inlineStr">
         <is>
-          <t>The next_light_check_at is set to a time that is at least 4 minutes 15 seconds and at most 5 minutes 45 seconds from the recorded time. (Reference: UC §4 step 5, FR-EXBOT-013.)</t>
+          <t>1. next_light_check_at is at least 4 minutes 15 seconds and at most 5 minutes 45 seconds from recorded time.
+2. Jitter within range [−45s, +45s].
+(Reference: UC §4 step 5, FR-EXBOT-013.)</t>
         </is>
       </c>
       <c r="F23" s="114" t="inlineStr">
@@ -15975,12 +16061,16 @@
       </c>
       <c r="D24" s="114" t="inlineStr">
         <is>
-          <t>Send a resume request while tracking HL API calls.</t>
+          <t>1. Start HL API monitoring.
+2. Send POST /api/exbot/resume.
+3. Check HL API logs.</t>
         </is>
       </c>
       <c r="E24" s="114" t="inlineStr">
         <is>
-          <t>Zero HL API calls are made during the resume operation. The light-check message is enqueued, but light-check itself makes no HL calls per BR-EXBOT-003. (Reference: UC §4, BR-EXBOT-003.)</t>
+          <t>1. Zero HL API calls during resume operation.
+2. Light-check message enqueued (separate worker makes no HL calls per BR-EXBOT-003).
+(Reference: UC §4, BR-EXBOT-003.)</t>
         </is>
       </c>
       <c r="F24" s="114" t="inlineStr">
@@ -16019,12 +16109,16 @@
       </c>
       <c r="D26" s="114" t="inlineStr">
         <is>
-          <t>Send a resume request for the bot. Read the audit log for the latest entry.</t>
+          <t>1. Send POST /api/exbot/resume.
+2. Query audit_log WHERE bot_id=X ORDER BY created_at DESC LIMIT 1.</t>
         </is>
       </c>
       <c r="E26" s="114" t="inlineStr">
         <is>
-          <t>The audit log contains an entry with the action "Bot resumed by investor", the bot ID, the user ID, and a timestamp matching the resume time. (Reference: UC §7 Postconditions.)</t>
+          <t>1. Audit log entry exists with action='Bot resumed by investor'.
+2. bot_id and user_wallet_address correct.
+3. created_at timestamp matches resume time.
+(Reference: UC §7 Postconditions.)</t>
         </is>
       </c>
       <c r="F26" s="114" t="inlineStr">
@@ -16051,12 +16145,16 @@
       </c>
       <c r="D27" s="114" t="inlineStr">
         <is>
-          <t>Send a resume request for the bot. Trigger a bot-scan cycle.</t>
+          <t>1. Send POST /api/exbot/resume.
+2. Trigger bot-scan cycle.
+3. Observe bot inclusion and scheduling.</t>
         </is>
       </c>
       <c r="E27" s="114" t="inlineStr">
         <is>
-          <t>The resumed bot with status='active' is included in the scan and receives a light-check message as scheduled. (Reference: UC §4 step 5, flows.md F-01.)</t>
+          <t>1. Resumed bot with status='active' included in scan.
+2. Bot receives light-check message as scheduled.
+(Reference: UC §4 step 5, flows.md F-01.)</t>
         </is>
       </c>
       <c r="F27" s="114" t="inlineStr">
@@ -16095,12 +16193,17 @@
       </c>
       <c r="D29" s="114" t="inlineStr">
         <is>
-          <t>Send a resume request but simulate a Lambda crash before the transaction commits.</t>
+          <t>1. Send POST /api/exbot/resume.
+2. Simulate Lambda crash before transaction commits.
+3. Query Aurora PostgreSQL.</t>
         </is>
       </c>
       <c r="E29" s="114" t="inlineStr">
         <is>
-          <t>Aurora PostgreSQL stays in the previous consistent state (status='paused'). No partial or inconsistent status value is left in the database. (Reference: Q3 resolved.)</t>
+          <t>1. Aurora PostgreSQL stays at previous consistent state (bots.status='paused').
+2. next_light_check_at unchanged.
+3. No partial state left in database.
+(Reference: Q3 resolved.)</t>
         </is>
       </c>
       <c r="F29" s="114" t="inlineStr">
@@ -16151,12 +16254,18 @@
       </c>
       <c r="D32" s="114" t="inlineStr">
         <is>
-          <t>Deliver the light-check message to the worker.</t>
+          <t>1. Deliver light-check message to worker.
+2. Worker evaluates bots.status='paused' at eligibility gate.
+3. Worker skips entire light-check.</t>
         </is>
       </c>
       <c r="E32" s="114" t="inlineStr">
         <is>
-          <t>The worker skips the entire light-check. No drift, range, or funding evaluation is run. No hedge-sync message is enqueued. The worker returns without error. (Reference: UC §6, FR-EXBOT-012.)</t>
+          <t>1. Worker skips all processing.
+2. No drift, range, or funding evaluation run.
+3. No hedge-sync message enqueued.
+4. Worker returns without error.
+(Reference: UC §6, FR-EXBOT-012.)</t>
         </is>
       </c>
       <c r="F32" s="114" t="inlineStr">
@@ -16183,12 +16292,15 @@
       </c>
       <c r="D33" s="114" t="inlineStr">
         <is>
-          <t>Deliver the pending light-check message to the worker.</t>
+          <t>1. Deliver pending light-check message to worker.
+2. Observe evaluation order.</t>
         </is>
       </c>
       <c r="E33" s="114" t="inlineStr">
         <is>
-          <t>The worker checks status='paused' at the eligibility gate before any other evaluation. The skip happens at the gate entry, not after partial work. (Reference: FR-EXBOT-012.)</t>
+          <t>1. Worker checks bots.status='paused' at gate entry BEFORE any other evaluation.
+2. Skip happens at gate, not after partial work.
+(Reference: FR-EXBOT-012.)</t>
         </is>
       </c>
       <c r="F33" s="114" t="inlineStr">
@@ -16215,12 +16327,16 @@
       </c>
       <c r="D34" s="114" t="inlineStr">
         <is>
-          <t>Deliver the hedge-sync message to the worker.</t>
+          <t>1. Deliver hedge-sync message to worker.
+2. Worker evaluates bots.status='paused'.</t>
         </is>
       </c>
       <c r="E34" s="114" t="inlineStr">
         <is>
-          <t>The worker does not submit any HL order. No hedge_legs records are modified. Hedge-sync is suppressed for paused bots. (Reference: UC §6.)</t>
+          <t>1. Worker does not submit any HL order.
+2. No hedge_legs records modified.
+3. Hedge-sync suppressed for paused bots.
+(Reference: UC §6.)</t>
         </is>
       </c>
       <c r="F34" s="114" t="inlineStr">
@@ -16247,12 +16363,18 @@
       </c>
       <c r="D35" s="114" t="inlineStr">
         <is>
-          <t>Let the scheduled deep-audit run.</t>
+          <t>1. Let scheduled deep-audit run.
+2. Deep-audit worker fetches clearinghouseState from HL.
+3. Verify hedge size, update margin status.</t>
         </is>
       </c>
       <c r="E35" s="114" t="inlineStr">
         <is>
-          <t>Deep-audit fetches the clearinghouse state from HL, verifies the hedge size matches the last known value, and updates the margin status. No anomaly is detected. (Reference: UC §6, FR-EXBOT-016.)</t>
+          <t>1. Deep-audit runs normally.
+2. hedge_legs.margin_status updated.
+3. No anomaly detected.
+4. bots.status='paused' unchanged.
+(Reference: UC §6, FR-EXBOT-016.)</t>
         </is>
       </c>
       <c r="F35" s="114" t="inlineStr">
@@ -16279,12 +16401,16 @@
       </c>
       <c r="D36" s="114" t="inlineStr">
         <is>
-          <t>Let the scheduled deep-audit run.</t>
+          <t>1. Let scheduled deep-audit run.
+2. Deep-audit worker runs at 1-hour interval.</t>
         </is>
       </c>
       <c r="E36" s="114" t="inlineStr">
         <is>
-          <t>Deep-audit runs at the 1-hour interval instead of the normal 6-hour interval. The worker fetches HL state and updates margin status. (Reference: FR-EXBOT-016.)</t>
+          <t>1. Deep-audit runs at 1-hour interval instead of 6-hour.
+2. Worker fetches HL state, updates margin status.
+3. High-risk cadence independent of pause state.
+(Reference: FR-EXBOT-016.)</t>
         </is>
       </c>
       <c r="F36" s="114" t="inlineStr">
@@ -16311,12 +16437,16 @@
       </c>
       <c r="D37" s="114" t="inlineStr">
         <is>
-          <t>Run the stop trigger evaluation for the paused bot.</t>
+          <t>1. Run stop trigger evaluation for paused bot.
+2. Observe monitoring behavior.</t>
         </is>
       </c>
       <c r="E37" s="114" t="inlineStr">
         <is>
-          <t>Even though light-check is skipped for paused bots, stop monitoring continues. A price-near-stop-audit message is enqueued when the mark price crosses the stop price. Stop monitoring is never suppressed. (Reference: FR-EXBOT-014.)</t>
+          <t>1. Stop monitoring continues.
+2. price-near-stop-audit message enqueued when mark price crosses stop price.
+3. Stop monitoring never suppressed.
+(Reference: FR-EXBOT-014.)</t>
         </is>
       </c>
       <c r="F37" s="114" t="inlineStr">
@@ -16343,12 +16473,16 @@
       </c>
       <c r="D38" s="114" t="inlineStr">
         <is>
-          <t>Let deep-audit run and detect the stuck stop trigger.</t>
+          <t>1. Let deep-audit run.
+2. Deep-audit detects stuck stop trigger.
+3. Observe transition.</t>
         </is>
       </c>
       <c r="E38" s="114" t="inlineStr">
         <is>
-          <t>The status changes from 'paused' to 'safe_mode'. The lifecycle_state stays at its pre-pause value. (Reference: FR-EXBOT-033, states.md.)</t>
+          <t>1. bots.status changes from 'paused' to 'safe_mode'.
+2. bots.lifecycle_state preserved.
+(Reference: FR-EXBOT-033, states.md.)</t>
         </is>
       </c>
       <c r="F38" s="114" t="inlineStr">
@@ -16375,12 +16509,15 @@
       </c>
       <c r="D39" s="114" t="inlineStr">
         <is>
-          <t>Run deep-audit and detect margin_status='critical'. Run the next deep-audit cycle while still paused and detect margin_status='critical' again.</t>
+          <t>1. Run deep-audit -&gt; detects margin_status='critical'.
+2. Run next deep-audit cycle while still paused -&gt; detects 'critical' again.</t>
         </is>
       </c>
       <c r="E39" s="114" t="inlineStr">
         <is>
-          <t>The status changes from 'paused' to 'safe_mode'. The lifecycle_state is preserved. (Reference: FR-EXBOT-050, FR-EXBOT-060.)</t>
+          <t>1. bots.status changes from 'paused' to 'safe_mode'.
+2. bots.lifecycle_state preserved.
+(Reference: FR-EXBOT-050, FR-EXBOT-060.)</t>
         </is>
       </c>
       <c r="F39" s="114" t="inlineStr">
@@ -16407,12 +16544,17 @@
       </c>
       <c r="D40" s="114" t="inlineStr">
         <is>
-          <t>Record the current count and values in rebalance_attempts and lp_operations. Send a pause request. Read the tables again.</t>
+          <t>1. Record current count in rebalance_attempts and lp_operations tables.
+2. Send POST /api/exbot/pause.
+3. Read tables again.</t>
         </is>
       </c>
       <c r="E40" s="114" t="inlineStr">
         <is>
-          <t>No new rows are inserted and no existing rows are modified in rebalance_attempts or lp_operations. All records are unchanged. (Reference: UC §3.)</t>
+          <t>1. No new rows inserted.
+2. No existing rows modified.
+3. All records unchanged.
+(Reference: UC §3.)</t>
         </is>
       </c>
       <c r="F40" s="114" t="inlineStr">
@@ -16451,12 +16593,17 @@
       </c>
       <c r="D42" s="114" t="inlineStr">
         <is>
-          <t>Trigger the bot-scan cron.</t>
+          <t>1. Send POST /api/exbot/resume.
+2. Trigger bot-scan cron.
+3. Observe bot inclusion.</t>
         </is>
       </c>
       <c r="E42" s="114" t="inlineStr">
         <is>
-          <t>The scan worker selects the bot with status='active' and schedules a light-check. The next_light_check_at is updated. (Reference: flows.md F-01.)</t>
+          <t>1. Scan worker selects bot with status='active'.
+2. light-check scheduled.
+3. next_light_check_at updated.
+(Reference: flows.md F-01.)</t>
         </is>
       </c>
       <c r="F42" s="114" t="inlineStr">
@@ -16495,12 +16642,16 @@
       </c>
       <c r="D44" s="114" t="inlineStr">
         <is>
-          <t>Have Investor B send a pause request for Investor A's bot.</t>
+          <t>1. Investor B sends POST /api/exbot/pause for Investor A's bot.
+2. Lambda verifies wallet ownership.</t>
         </is>
       </c>
       <c r="E44" s="114" t="inlineStr">
         <is>
-          <t>The request is rejected before any Aurora PostgreSQL mutation. The API returns HTTP 403 or HTTP 404. No audit log entry is written for the unauthorized attempt. (Reference: FR-EXBOT-001.)</t>
+          <t>1. Request rejected before Aurora PostgreSQL mutation.
+2. API returns HTTP 403 or HTTP 404.
+3. No audit log entry for unauthorized attempt.
+(Reference: FR-EXBOT-001.)</t>
         </is>
       </c>
       <c r="F44" s="114" t="inlineStr">
@@ -16527,12 +16678,16 @@
       </c>
       <c r="D45" s="114" t="inlineStr">
         <is>
-          <t>Record the time before sending a pause request. Send the pause request. Record the time when the HTTP response is received.</t>
+          <t>1. Record time before sending pause request.
+2. Send POST /api/exbot/pause.
+3. Record time when HTTP response received.</t>
         </is>
       </c>
       <c r="E45" s="114" t="inlineStr">
         <is>
-          <t>The operation completes within the target SLA (a fast operation with zero HL API calls and zero vault calls). (Reference: NFR.)</t>
+          <t>1. Operation completes within target SLA (fast operation, zero HL API calls, zero vault calls).
+2. Expected: &lt;100ms (API latency NFR).
+(Reference: NFR.)</t>
         </is>
       </c>
       <c r="F45" s="114" t="inlineStr">

</xml_diff>